<commit_message>
stage3: import wizard + anomaly rules (R6 fixed to personNo intersection) + pending pool with batch resolve
</commit_message>
<xml_diff>
--- a/public/samples/获奖公示模板.xlsx
+++ b/public/samples/获奖公示模板.xlsx
@@ -398,17 +398,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I5"/>
-  <cols>
-    <col min="1" max="1" width="42.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="32.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="52.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -441,13 +430,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>基于多模态感知的智能巡检系统·校园安全场景</v>
+        <v>柔性传感与智能康复设备·校园安全场景</v>
       </c>
       <c r="B2">
         <v>2026</v>
       </c>
       <c r="C2" t="str">
-        <v>机械与动力学院</v>
+        <v>化学与分子科学学院</v>
       </c>
       <c r="D2" t="str">
         <v>中国国际大学生创新大赛</v>
@@ -462,10 +451,10 @@
         <v>https://example.edu.cn/awards/sample/valid</v>
       </c>
       <c r="H2" t="str">
-        <v>2023000437</v>
+        <v>2023000463</v>
       </c>
       <c r="I2" t="str">
-        <v>黄宇轩</v>
+        <v>陈宇轩</v>
       </c>
     </row>
     <row r="3">

</xml_diff>